<commit_message>
v2: vigas aereas, losa, correas, colores por objeto, unidades metricas, autor y presentacion
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013BqHCBCBMxPVbrFpj9LrZE
</commit_message>
<xml_diff>
--- a/PARAM_2026-2_ACT03_GRUPO##_MATRIZ_FINAL.xlsx
+++ b/PARAM_2026-2_ACT03_GRUPO##_MATRIZ_FINAL.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="331">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="354">
   <si>
     <t xml:space="preserve">ACTIVIDAD 3 - BIM PARAMETRIZACION | MATRIZ FINAL | HOJA 1: PACIENTE Y OBJETOS</t>
   </si>
@@ -79,10 +79,16 @@
     <t xml:space="preserve">ISO 19650 (gestion de informacion y nomenclatura), IFC 4 (clases de intercambio), Uniclass 2015 tabla EF, NSR-10 Titulos B y C.</t>
   </si>
   <si>
-    <t xml:space="preserve">Grupo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRUPO ## (completar numero y nombres de los integrantes en la columna Responsable)</t>
+    <t xml:space="preserve">Autor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luis David Arroyo Anaya - Maestria en Patologia de la Construccion, Facultad de Ingenieria Civil, Universidad Santo Tomas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colores en el modelo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zapatas gris, columnas azul, vigas de cimentacion verde, vigas aereas naranja, losa amarilla (transparente), correas rojo.</t>
   </si>
   <si>
     <t xml:space="preserve">N.</t>
@@ -157,9 +163,6 @@
     <t xml:space="preserve">EF_25_10</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 2 (completar)</t>
-  </si>
-  <si>
     <t xml:space="preserve">VCI</t>
   </si>
   <si>
@@ -178,9 +181,6 @@
     <t xml:space="preserve">IfcBeam.BEAM</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 3 (completar)</t>
-  </si>
-  <si>
     <t xml:space="preserve">COR</t>
   </si>
   <si>
@@ -190,7 +190,7 @@
     <t xml:space="preserve">Armazon estructural - correas (Structural Framing)</t>
   </si>
   <si>
-    <t xml:space="preserve">P89_COR_Perfil_C_PHR (cargable, familia propia separada de la viga)</t>
+    <t xml:space="preserve">P89_COR_Correa_PHR (cargable, familia propia; seccion rectangular equivalente 60x160 mm)</t>
   </si>
   <si>
     <t xml:space="preserve">PHR C 160x60x20 e = 1,50 mm</t>
@@ -202,10 +202,43 @@
     <t xml:space="preserve">EF_30_10</t>
   </si>
   <si>
-    <t xml:space="preserve">Integrante 4 (completar)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Celdas amarillas: datos que el grupo debe completar.</t>
+    <t xml:space="preserve">ELEMENTOS COMPLEMENTARIOS DEL MODELO (no son objetos evaluados: llevan solo los 5 parametros comunes PAC_ para mantener la consistencia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VIG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Viga aerea de concreto (VG)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P89_VIG_Viga_Aerea: VG-30x50, VG-20x50, VG-12x50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa maciza de entrepiso N+3,05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Suelos estructurales (Floors)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Losa maciza P89 e=0,15 m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IfcSlab.FLOOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EF_30_20</t>
   </si>
   <si>
     <t xml:space="preserve">HOJA 2: MATRIZ MAESTRA DE PARAMETROS IMPLEMENTADOS (fuente unica para el modelo y el Schedule)</t>
@@ -277,9 +310,6 @@
     <t xml:space="preserve">Datos de identidad</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
-  </si>
-  <si>
     <t xml:space="preserve">85472c8c-6490-518b-a29e-b885faa36d93</t>
   </si>
   <si>
@@ -694,10 +724,25 @@
     <t xml:space="preserve">e = 1,50 mm</t>
   </si>
   <si>
+    <t xml:space="preserve">VG-30x50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VG-20x50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VG-12x50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IfcSlab.FLOOR | EF_30_20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VERIFICAR espesor y refuerzo (el DWG no rotula el espesor)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total concreto zapatas</t>
   </si>
   <si>
-    <t xml:space="preserve">Cantidad segun plano: conteo de etiquetas y elementos en la Planta de Cimentaciones del DWG P89-2022 (VC = tramos entre columnas sobre un mismo eje; correas: 12 a ~1,00 m). Cantidad en Schedule (amarillo): copiar el conteo del Schedule P89_ACT03_VALIDACION.</t>
+    <t xml:space="preserve">Cantidad segun plano: conteo de etiquetas y elementos en la Planta de Cimentaciones del DWG P89-2022 (VC = tramos entre columnas sobre un mismo eje; correas: 24 a ~1,00 m en 3 zonas de cubierta; VG = tramos de las plantas N+3,05 y N+6,05; losa = 2 paños). Cantidad en Schedule (amarillo): copiar el conteo del Schedule P89_ACT03_VALIDACION.</t>
   </si>
   <si>
     <t xml:space="preserve">HOJA 4: ESTRATEGIA COMUN DE PARAMETRIZACION Y JUSTIFICACION</t>
@@ -793,6 +838,24 @@
     <t xml:space="preserve">Conclusion de la revision grupal: duplicar nativos produce valores que pueden contradecirse con la geometria.</t>
   </si>
   <si>
+    <t xml:space="preserve">Elementos complementarios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vigas aereas VG (N+3,05 y N+6,05) y losa maciza de entrepiso: se modelan para completar el paciente y llevan solo los 5 parametros comunes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Muestran que la estrategia comun se puede extender a cualquier elemento nuevo sin crear parametros nuevos ni duplicados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Colores por objeto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un material por objeto: zapata gris, columna azul, VC verde, VG naranja, losa amarilla, correa roja. Vista '3D P89 ACT03 - Colores por objeto'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Permite reconocer cada objeto del paciente en el modelo y en el video; el material tambien queda en el parametro nativo Material estructural.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Validacion</t>
   </si>
   <si>
@@ -1037,6 +1100,12 @@
   </si>
   <si>
     <t xml:space="preserve">PAC_Norma_Diseno esta lleno en Informacion de proyecto.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Las vigas aereas VG y la losa tienen llenos los 5 parametros comunes en el Schedule.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espesor de la losa maciza (0,15 m) confirmado con la memoria de calculo.</t>
   </si>
   <si>
     <t xml:space="preserve">El archivo Excel no tiene macros (.xlsx).</t>
@@ -1156,14 +1225,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFDDEBF7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE2EFDA"/>
-        <bgColor rgb="FFDDEBF7"/>
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
@@ -1253,16 +1322,12 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1301,7 +1366,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1310,6 +1375,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1626,7 +1695,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1727,164 +1796,238 @@
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
     </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="s">
+    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+    </row>
+    <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="B10" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="C10" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I9" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="5" t="s">
+      <c r="H10" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="I10" s="4" t="s">
         <v>21</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="I11" s="5" t="s">
         <v>29</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>42</v>
+      <c r="I12" s="5" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I13" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B14" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F13" s="5" t="s">
+      <c r="F14" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G13" s="5" t="s">
+      <c r="G14" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="H13" s="5" t="s">
+      <c r="H14" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="I13" s="6" t="s">
+      <c r="I14" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
+    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="s">
         <v>51</v>
       </c>
+      <c r="B17" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F18" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="I18" s="5" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="B4:I4"/>
     <mergeCell ref="B5:I5"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B7:I7"/>
+    <mergeCell ref="B8:I8"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1922,7 +2065,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1943,1059 +2086,1059 @@
       <c r="R1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="8"/>
-      <c r="N2" s="8"/>
-      <c r="O2" s="8"/>
-      <c r="P2" s="8"/>
-      <c r="Q2" s="8"/>
-      <c r="R2" s="8"/>
+      <c r="A2" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
+      <c r="M2" s="6"/>
+      <c r="N2" s="6"/>
+      <c r="O2" s="6"/>
+      <c r="P2" s="6"/>
+      <c r="Q2" s="6"/>
+      <c r="R2" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>54</v>
+        <v>65</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>57</v>
+        <v>68</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>59</v>
+        <v>70</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="L4" s="4" t="s">
         <v>43</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>60</v>
+        <v>71</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>61</v>
+        <v>72</v>
       </c>
       <c r="O4" s="4" t="s">
-        <v>62</v>
+        <v>73</v>
       </c>
       <c r="P4" s="4" t="s">
-        <v>63</v>
+        <v>74</v>
       </c>
       <c r="Q4" s="4" t="s">
-        <v>64</v>
+        <v>75</v>
       </c>
       <c r="R4" s="4" t="s">
-        <v>65</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F5" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H5" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I5" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J5" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="L5" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M5" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="N5" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="O5" s="9" t="s">
-        <v>76</v>
-      </c>
-      <c r="P5" s="9" t="s">
+      <c r="B5" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="C5" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="R5" s="6"/>
+      <c r="D5" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F5" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H5" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J5" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="K5" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="L5" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="M5" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>86</v>
+      </c>
+      <c r="P5" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="Q5" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="R5" s="8"/>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="9" t="s">
+      <c r="B6" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>90</v>
+      </c>
+      <c r="D6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="E6" s="7" t="s">
         <v>80</v>
       </c>
-      <c r="D6" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F6" s="9" t="s">
+      <c r="F6" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="K6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="L6" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="M6" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="N6" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="P6" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q6" s="7" t="s">
+        <v>94</v>
+      </c>
+      <c r="R6" s="8"/>
+    </row>
+    <row r="7" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>95</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="K7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>85</v>
+      </c>
+      <c r="N7" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="P7" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="Q7" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="R7" s="8"/>
+    </row>
+    <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F8" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="G6" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H6" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="L6" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M6" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="N6" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="O6" s="9" t="s">
+      <c r="G8" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="P6" s="9" t="s">
+      <c r="H8" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="Q6" s="9" t="s">
+      <c r="I8" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="R6" s="6"/>
-    </row>
-    <row r="7" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="9" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="9" t="s">
+      <c r="J8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="K8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="M8" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="N8" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O8" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="P8" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="Q8" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="R8" s="8"/>
+    </row>
+    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="K9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="M9" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="N9" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="O9" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="P9" s="7" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q9" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="R9" s="8"/>
+    </row>
+    <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C7" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>87</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="F7" s="9" t="s">
+      <c r="N10" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="O10" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="P10" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q10" s="9" t="s">
+        <v>121</v>
+      </c>
+      <c r="R10" s="8"/>
+    </row>
+    <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E11" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J11" s="10"/>
+      <c r="K11" s="10"/>
+      <c r="L11" s="10"/>
+      <c r="M11" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N11" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O11" s="10" t="s">
+        <v>129</v>
+      </c>
+      <c r="P11" s="10" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q11" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="R11" s="8"/>
+    </row>
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>132</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E12" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J12" s="10"/>
+      <c r="K12" s="10"/>
+      <c r="L12" s="10"/>
+      <c r="M12" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N12" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O12" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="P12" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="Q12" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="R12" s="8"/>
+    </row>
+    <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>139</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>140</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="J13" s="10"/>
+      <c r="K13" s="10"/>
+      <c r="L13" s="10"/>
+      <c r="M13" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N13" s="10" t="s">
+        <v>141</v>
+      </c>
+      <c r="O13" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="P13" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="Q13" s="10" t="s">
+        <v>144</v>
+      </c>
+      <c r="R13" s="8"/>
+    </row>
+    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="10" t="s">
+        <v>145</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>146</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E14" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F14" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I14" s="10"/>
+      <c r="J14" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="K14" s="10"/>
+      <c r="L14" s="10"/>
+      <c r="M14" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N14" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O14" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="P14" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="Q14" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="R14" s="8"/>
+    </row>
+    <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E15" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F15" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="G7" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="L7" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M7" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="N7" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="O7" s="9" t="s">
-        <v>89</v>
-      </c>
-      <c r="P7" s="9" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q7" s="9" t="s">
+      <c r="G15" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I15" s="10"/>
+      <c r="J15" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="K15" s="10"/>
+      <c r="L15" s="10"/>
+      <c r="M15" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>152</v>
+      </c>
+      <c r="P15" s="10" t="s">
+        <v>153</v>
+      </c>
+      <c r="Q15" s="10" t="s">
+        <v>154</v>
+      </c>
+      <c r="R15" s="8"/>
+    </row>
+    <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>155</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E16" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F16" s="10" t="s">
         <v>91</v>
       </c>
-      <c r="R7" s="6"/>
-    </row>
-    <row r="8" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="9" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>92</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>93</v>
-      </c>
-      <c r="D8" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="9" t="s">
-        <v>70</v>
-      </c>
-      <c r="G8" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="L8" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M8" s="9" t="s">
-        <v>94</v>
-      </c>
-      <c r="N8" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="O8" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="P8" s="9" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q8" s="9" t="s">
-        <v>97</v>
-      </c>
-      <c r="R8" s="6"/>
-    </row>
-    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="9" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>99</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>68</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>69</v>
-      </c>
-      <c r="F9" s="9" t="s">
+      <c r="G16" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I16" s="10"/>
+      <c r="J16" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="K16" s="10"/>
+      <c r="L16" s="10"/>
+      <c r="M16" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="N16" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O16" s="10" t="s">
+        <v>157</v>
+      </c>
+      <c r="P16" s="10" t="s">
+        <v>158</v>
+      </c>
+      <c r="Q16" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="R16" s="8"/>
+    </row>
+    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I17" s="10"/>
+      <c r="J17" s="10"/>
+      <c r="K17" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="L17" s="10"/>
+      <c r="M17" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N17" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O17" s="10" t="s">
+        <v>161</v>
+      </c>
+      <c r="P17" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="Q17" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="R17" s="8"/>
+    </row>
+    <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="10" t="s">
+        <v>163</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>164</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E18" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F18" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="G9" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H9" s="9" t="s">
-        <v>72</v>
-      </c>
-      <c r="I9" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="L9" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="M9" s="9" t="s">
-        <v>100</v>
-      </c>
-      <c r="N9" s="9" t="s">
-        <v>75</v>
-      </c>
-      <c r="O9" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="P9" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="Q9" s="9" t="s">
-        <v>103</v>
-      </c>
-      <c r="R9" s="6"/>
-    </row>
-    <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>104</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>105</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>69</v>
-      </c>
-      <c r="F10" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>107</v>
-      </c>
-      <c r="H10" s="10" t="s">
-        <v>108</v>
-      </c>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="N10" s="10" t="s">
-        <v>75</v>
-      </c>
-      <c r="O10" s="10" t="s">
-        <v>109</v>
-      </c>
-      <c r="P10" s="10" t="s">
-        <v>110</v>
-      </c>
-      <c r="Q10" s="10" t="s">
-        <v>111</v>
-      </c>
-      <c r="R10" s="6"/>
-    </row>
-    <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>112</v>
-      </c>
-      <c r="C11" s="11" t="s">
-        <v>113</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E11" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F11" s="11" t="s">
+      <c r="G18" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I18" s="10"/>
+      <c r="J18" s="10"/>
+      <c r="K18" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="N18" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O18" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="P18" s="10" t="s">
+        <v>166</v>
+      </c>
+      <c r="Q18" s="10" t="s">
+        <v>167</v>
+      </c>
+      <c r="R18" s="8"/>
+    </row>
+    <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>169</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E19" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I19" s="10"/>
+      <c r="J19" s="10"/>
+      <c r="K19" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="N19" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O19" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="P19" s="10" t="s">
+        <v>171</v>
+      </c>
+      <c r="Q19" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="R19" s="8"/>
+    </row>
+    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>173</v>
+      </c>
+      <c r="D20" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="F20" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H20" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I20" s="10"/>
+      <c r="J20" s="10"/>
+      <c r="K20" s="10"/>
+      <c r="L20" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="M20" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="N20" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O20" s="10" t="s">
+        <v>174</v>
+      </c>
+      <c r="P20" s="10" t="s">
+        <v>175</v>
+      </c>
+      <c r="Q20" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="R20" s="8"/>
+    </row>
+    <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>176</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>177</v>
+      </c>
+      <c r="D21" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E21" s="10" t="s">
+        <v>178</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="H21" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="I21" s="10"/>
+      <c r="J21" s="10"/>
+      <c r="K21" s="10"/>
+      <c r="L21" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="M21" s="10" t="s">
+        <v>128</v>
+      </c>
+      <c r="N21" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O21" s="10" t="s">
+        <v>179</v>
+      </c>
+      <c r="P21" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q21" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="R21" s="8"/>
+    </row>
+    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>182</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="E22" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="F22" s="10" t="s">
         <v>81</v>
       </c>
-      <c r="G11" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H11" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N11" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O11" s="11" t="s">
-        <v>119</v>
-      </c>
-      <c r="P11" s="11" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q11" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="R11" s="6"/>
-    </row>
-    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="11" t="s">
-        <v>122</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E12" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F12" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G12" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H12" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I12" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N12" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O12" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="P12" s="11" t="s">
-        <v>125</v>
-      </c>
-      <c r="Q12" s="11" t="s">
+      <c r="G22" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="R12" s="6"/>
-    </row>
-    <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="11" t="s">
+      <c r="H22" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="I22" s="10"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10" t="s">
+        <v>84</v>
+      </c>
+      <c r="M22" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="D13" s="11" t="s">
-        <v>129</v>
-      </c>
-      <c r="E13" s="11" t="s">
-        <v>130</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H13" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I13" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N13" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="O13" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="P13" s="11" t="s">
-        <v>133</v>
-      </c>
-      <c r="Q13" s="11" t="s">
-        <v>134</v>
-      </c>
-      <c r="R13" s="6"/>
-    </row>
-    <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="11" t="s">
-        <v>135</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>136</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F14" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H14" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I14" s="11"/>
-      <c r="J14" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N14" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O14" s="11" t="s">
-        <v>137</v>
-      </c>
-      <c r="P14" s="11" t="s">
-        <v>138</v>
-      </c>
-      <c r="Q14" s="11" t="s">
-        <v>139</v>
-      </c>
-      <c r="R14" s="6"/>
-    </row>
-    <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="11" t="s">
-        <v>140</v>
-      </c>
-      <c r="C15" s="11" t="s">
-        <v>141</v>
-      </c>
-      <c r="D15" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E15" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G15" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H15" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I15" s="11"/>
-      <c r="J15" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N15" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O15" s="11" t="s">
-        <v>142</v>
-      </c>
-      <c r="P15" s="11" t="s">
-        <v>143</v>
-      </c>
-      <c r="Q15" s="11" t="s">
-        <v>144</v>
-      </c>
-      <c r="R15" s="6"/>
-    </row>
-    <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>146</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F16" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H16" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="N16" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O16" s="11" t="s">
-        <v>147</v>
-      </c>
-      <c r="P16" s="11" t="s">
-        <v>148</v>
-      </c>
-      <c r="Q16" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="R16" s="6"/>
-    </row>
-    <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>149</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>150</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E17" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F17" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G17" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H17" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I17" s="11"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N17" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O17" s="11" t="s">
-        <v>151</v>
-      </c>
-      <c r="P17" s="11" t="s">
-        <v>152</v>
-      </c>
-      <c r="Q17" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="R17" s="6"/>
-    </row>
-    <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>153</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E18" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F18" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G18" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H18" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I18" s="11"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="N18" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O18" s="11" t="s">
-        <v>155</v>
-      </c>
-      <c r="P18" s="11" t="s">
-        <v>156</v>
-      </c>
-      <c r="Q18" s="11" t="s">
-        <v>157</v>
-      </c>
-      <c r="R18" s="6"/>
-    </row>
-    <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="11" t="s">
-        <v>158</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>159</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F19" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H19" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I19" s="11"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="N19" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O19" s="11" t="s">
-        <v>160</v>
-      </c>
-      <c r="P19" s="11" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q19" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="R19" s="6"/>
-    </row>
-    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="11" t="s">
-        <v>162</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>163</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="F20" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H20" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I20" s="11"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="M20" s="11" t="s">
-        <v>74</v>
-      </c>
-      <c r="N20" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O20" s="11" t="s">
-        <v>164</v>
-      </c>
-      <c r="P20" s="11" t="s">
-        <v>165</v>
-      </c>
-      <c r="Q20" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="R20" s="6"/>
-    </row>
-    <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>166</v>
-      </c>
-      <c r="C21" s="11" t="s">
-        <v>167</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E21" s="11" t="s">
-        <v>168</v>
-      </c>
-      <c r="F21" s="11" t="s">
-        <v>81</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H21" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="M21" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N21" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O21" s="11" t="s">
-        <v>169</v>
-      </c>
-      <c r="P21" s="11" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q21" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="R21" s="6"/>
-    </row>
-    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>171</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>172</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>115</v>
-      </c>
-      <c r="F22" s="11" t="s">
-        <v>70</v>
-      </c>
-      <c r="G22" s="11" t="s">
-        <v>116</v>
-      </c>
-      <c r="H22" s="11" t="s">
-        <v>117</v>
-      </c>
-      <c r="I22" s="11"/>
-      <c r="J22" s="11"/>
-      <c r="K22" s="11"/>
-      <c r="L22" s="11" t="s">
-        <v>73</v>
-      </c>
-      <c r="M22" s="11" t="s">
-        <v>118</v>
-      </c>
-      <c r="N22" s="11" t="s">
-        <v>75</v>
-      </c>
-      <c r="O22" s="11" t="s">
-        <v>173</v>
-      </c>
-      <c r="P22" s="11" t="s">
-        <v>174</v>
-      </c>
-      <c r="Q22" s="11" t="s">
-        <v>175</v>
-      </c>
-      <c r="R22" s="6"/>
+      <c r="N22" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="O22" s="10" t="s">
+        <v>183</v>
+      </c>
+      <c r="P22" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q22" s="10" t="s">
+        <v>185</v>
+      </c>
+      <c r="R22" s="8"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
-        <v>176</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="11" t="n">
         <f aca="false">COUNTIF(G5:G22,"Comun")</f>
         <v>5</v>
       </c>
-      <c r="C24" s="13" t="s">
-        <v>177</v>
+      <c r="C24" s="12" t="s">
+        <v>187</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B25" s="12" t="n">
+      <c r="B25" s="11" t="n">
         <f aca="false">COUNTIF(G5:G22,"Particular")</f>
         <v>12</v>
       </c>
-      <c r="C25" s="13" t="s">
-        <v>178</v>
+      <c r="C25" s="12" t="s">
+        <v>188</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="12" t="n">
+      <c r="B26" s="11" t="n">
         <f aca="false">COUNTIFS(G5:G22,"Particular",I5:I22,"X")</f>
         <v>3</v>
       </c>
-      <c r="C26" s="13" t="s">
-        <v>179</v>
+      <c r="C26" s="12" t="s">
+        <v>189</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="12" t="n">
+      <c r="B27" s="11" t="n">
         <f aca="false">COUNTIFS(G5:G22,"Particular",J5:J22,"X")</f>
         <v>3</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>180</v>
+      <c r="C27" s="12" t="s">
+        <v>190</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="12" t="n">
+      <c r="B28" s="11" t="n">
         <f aca="false">COUNTIFS(G5:G22,"Particular",K5:K22,"X")</f>
         <v>3</v>
       </c>
-      <c r="C28" s="13" t="s">
-        <v>181</v>
+      <c r="C28" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B29" s="12" t="n">
+      <c r="B29" s="11" t="n">
         <f aca="false">COUNTIFS(G5:G22,"Particular",L5:L22,"X")</f>
         <v>3</v>
       </c>
-      <c r="C29" s="13" t="s">
-        <v>182</v>
+      <c r="C29" s="12" t="s">
+        <v>192</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B30" s="12" t="n">
+      <c r="B30" s="11" t="n">
         <f aca="false">B24+B26</f>
         <v>8</v>
       </c>
-      <c r="C30" s="13" t="s">
-        <v>183</v>
+      <c r="C30" s="12" t="s">
+        <v>193</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="12" t="n">
+      <c r="B31" s="11" t="n">
         <f aca="false">SUMPRODUCT((COUNTIF(B5:B22,B5:B22)&gt;1)*1)</f>
         <v>0</v>
       </c>
-      <c r="C31" s="13" t="s">
-        <v>184</v>
+      <c r="C31" s="12" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="12" t="n">
+      <c r="B32" s="11" t="n">
         <f aca="false">COUNTIF(N5:N22,"&lt;&gt;-")</f>
         <v>1</v>
       </c>
-      <c r="C32" s="13" t="s">
-        <v>185</v>
+      <c r="C32" s="12" t="s">
+        <v>195</v>
       </c>
     </row>
   </sheetData>
@@ -3020,7 +3163,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M15"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="8"/>
@@ -3038,7 +3181,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>186</v>
+        <v>196</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3054,346 +3197,346 @@
       <c r="M1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="s">
-        <v>187</v>
-      </c>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
+      <c r="A2" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+      <c r="L2" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>189</v>
+        <v>199</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>191</v>
+        <v>201</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>192</v>
+        <v>202</v>
       </c>
       <c r="I4" s="4" t="s">
-        <v>193</v>
+        <v>203</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>194</v>
+        <v>204</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>195</v>
+        <v>205</v>
       </c>
       <c r="L4" s="4" t="s">
-        <v>196</v>
+        <v>206</v>
       </c>
       <c r="M4" s="4" t="s">
-        <v>197</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="C5" s="14" t="n">
+        <v>208</v>
+      </c>
+      <c r="C5" s="13" t="n">
         <v>1.3</v>
       </c>
-      <c r="D5" s="14" t="n">
+      <c r="D5" s="13" t="n">
         <v>0.35</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F5" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F5" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>201</v>
+        <v>210</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I5" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C5,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D5,"0.00"),".",",")</f>
         <v>1,30x0,35</v>
       </c>
-      <c r="J5" s="16" t="n">
+      <c r="J5" s="15" t="n">
         <f aca="false">C5*C5*D5</f>
         <v>0.5915</v>
       </c>
-      <c r="K5" s="15" t="n">
+      <c r="K5" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="L5" s="6"/>
-      <c r="M5" s="17" t="n">
+      <c r="L5" s="8"/>
+      <c r="M5" s="16" t="n">
         <f aca="false">J5*K5</f>
         <v>7.098</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="C6" s="14" t="n">
+        <v>212</v>
+      </c>
+      <c r="C6" s="13" t="n">
         <v>1.6</v>
       </c>
-      <c r="D6" s="14" t="n">
+      <c r="D6" s="13" t="n">
         <v>0.35</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F6" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F6" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>201</v>
+        <v>210</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I6" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C6,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D6,"0.00"),".",",")</f>
         <v>1,60x0,35</v>
       </c>
-      <c r="J6" s="16" t="n">
+      <c r="J6" s="15" t="n">
         <f aca="false">C6*C6*D6</f>
         <v>0.896</v>
       </c>
-      <c r="K6" s="15" t="n">
+      <c r="K6" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="L6" s="6"/>
-      <c r="M6" s="17" t="n">
+      <c r="L6" s="8"/>
+      <c r="M6" s="16" t="n">
         <f aca="false">J6*K6</f>
         <v>3.584</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="C7" s="14" t="n">
+        <v>213</v>
+      </c>
+      <c r="C7" s="13" t="n">
         <v>1.7</v>
       </c>
-      <c r="D7" s="14" t="n">
+      <c r="D7" s="13" t="n">
         <v>0.35</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F7" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F7" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>201</v>
+        <v>210</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I7" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C7,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D7,"0.00"),".",",")</f>
         <v>1,70x0,35</v>
       </c>
-      <c r="J7" s="16" t="n">
+      <c r="J7" s="15" t="n">
         <f aca="false">C7*C7*D7</f>
         <v>1.0115</v>
       </c>
-      <c r="K7" s="15" t="n">
+      <c r="K7" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="L7" s="6"/>
-      <c r="M7" s="17" t="n">
+      <c r="L7" s="8"/>
+      <c r="M7" s="16" t="n">
         <f aca="false">J7*K7</f>
         <v>3.0345</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="C8" s="14" t="n">
+        <v>214</v>
+      </c>
+      <c r="C8" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="D8" s="14" t="n">
+      <c r="D8" s="13" t="n">
         <v>0.3</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F8" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F8" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>201</v>
+        <v>215</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I8" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C8,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D8,"0.00"),".",",")</f>
         <v>0,30x0,30</v>
       </c>
-      <c r="J8" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="K8" s="15" t="n">
+      <c r="J8" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K8" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="L8" s="6"/>
+      <c r="L8" s="8"/>
       <c r="M8" s="5" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C9" s="14" t="n">
+        <v>216</v>
+      </c>
+      <c r="C9" s="13" t="n">
         <v>0.25</v>
       </c>
-      <c r="D9" s="14" t="n">
+      <c r="D9" s="13" t="n">
         <v>0.4</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F9" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F9" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>201</v>
+        <v>215</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I9" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C9,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D9,"0.00"),".",",")</f>
         <v>0,25x0,40</v>
       </c>
-      <c r="J9" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="K9" s="15" t="n">
+      <c r="J9" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K9" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="L9" s="6"/>
+      <c r="L9" s="8"/>
       <c r="M9" s="5" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="C10" s="14" t="n">
+        <v>217</v>
+      </c>
+      <c r="C10" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="D10" s="14" t="n">
+      <c r="D10" s="13" t="n">
         <v>0.25</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F10" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F10" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>201</v>
+        <v>215</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I10" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C10,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D10,"0.00"),".",",")</f>
         <v>0,40x0,25</v>
       </c>
-      <c r="J10" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="K10" s="15" t="n">
+      <c r="J10" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K10" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="L10" s="6"/>
+      <c r="L10" s="8"/>
       <c r="M10" s="5" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="C11" s="14" t="n">
+        <v>218</v>
+      </c>
+      <c r="C11" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="D11" s="14" t="n">
+      <c r="D11" s="13" t="n">
         <v>0.3</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="F11" s="15" t="n">
+        <v>209</v>
+      </c>
+      <c r="F11" s="14" t="n">
         <v>21</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="H11" s="6" t="s">
-        <v>201</v>
+        <v>219</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>211</v>
       </c>
       <c r="I11" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C11,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D11,"0.00"),".",",")</f>
         <v>0,30x0,30</v>
       </c>
-      <c r="J11" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="K11" s="15" t="n">
+      <c r="J11" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K11" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="L11" s="6"/>
+      <c r="L11" s="8"/>
       <c r="M11" s="5" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3401,53 +3544,212 @@
         <v>43</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="C12" s="14" t="n">
+        <v>220</v>
+      </c>
+      <c r="C12" s="13" t="n">
         <v>0.06</v>
       </c>
-      <c r="D12" s="14" t="n">
+      <c r="D12" s="13" t="n">
         <v>0.16</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="F12" s="18" t="n">
+        <v>221</v>
+      </c>
+      <c r="F12" s="17" t="n">
         <v>340</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>212</v>
+        <v>222</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>213</v>
+        <v>223</v>
       </c>
       <c r="I12" s="5" t="str">
         <f aca="false">SUBSTITUTE(TEXT(C12,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D12,"0.00"),".",",")</f>
         <v>0,06x0,16</v>
       </c>
-      <c r="J12" s="16" t="s">
-        <v>75</v>
-      </c>
-      <c r="K12" s="15" t="n">
-        <v>12</v>
-      </c>
-      <c r="L12" s="6"/>
+      <c r="J12" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K12" s="14" t="n">
+        <v>24</v>
+      </c>
+      <c r="L12" s="8"/>
       <c r="M12" s="5" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="I13" s="19" t="s">
-        <v>214</v>
-      </c>
-      <c r="M13" s="20" t="n">
-        <f aca="false">SUM(M5:M12)</f>
+      <c r="A13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F13" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="I13" s="5" t="str">
+        <f aca="false">SUBSTITUTE(TEXT(C13,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D13,"0.00"),".",",")</f>
+        <v>0,30x0,50</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K13" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="L13" s="8"/>
+      <c r="M13" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="C14" s="13" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F14" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="G14" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="I14" s="5" t="str">
+        <f aca="false">SUBSTITUTE(TEXT(C14,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D14,"0.00"),".",",")</f>
+        <v>0,20x0,50</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K14" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="L14" s="8"/>
+      <c r="M14" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="13" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D15" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F15" s="14" t="n">
+        <v>21</v>
+      </c>
+      <c r="G15" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>211</v>
+      </c>
+      <c r="I15" s="5" t="str">
+        <f aca="false">SUBSTITUTE(TEXT(C15,"0.00"),".",",")&amp;"x"&amp;SUBSTITUTE(TEXT(D15,"0.00"),".",",")</f>
+        <v>0,12x0,50</v>
+      </c>
+      <c r="J15" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="K15" s="14" t="n">
+        <v>19</v>
+      </c>
+      <c r="L15" s="8"/>
+      <c r="M15" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="H16" s="8" t="s">
+        <v>228</v>
+      </c>
+      <c r="I16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="K16" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I17" s="18" t="s">
+        <v>229</v>
+      </c>
+      <c r="M17" s="19" t="n">
+        <f aca="false">SUM(M5:M16)</f>
         <v>13.7165</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="s">
-        <v>215</v>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="20" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
@@ -3471,7 +3773,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -3481,130 +3783,152 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>216</v>
+        <v>231</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>217</v>
+        <v>232</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>218</v>
+        <v>233</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>219</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>221</v>
+        <v>236</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>222</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>223</v>
+        <v>238</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>225</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>226</v>
+        <v>241</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>227</v>
+        <v>242</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>228</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>229</v>
+        <v>244</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>230</v>
+        <v>245</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>231</v>
+        <v>246</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>249</v>
+        <v>264</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -3637,7 +3961,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>250</v>
+        <v>271</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3645,332 +3969,332 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>251</v>
+        <v>272</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>252</v>
+        <v>273</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>253</v>
+        <v>274</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>254</v>
+        <v>275</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>255</v>
+        <v>276</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>257</v>
+        <v>278</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>258</v>
+        <v>279</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>259</v>
+        <v>280</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>260</v>
+        <v>281</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>261</v>
+        <v>282</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>262</v>
+        <v>283</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>263</v>
+        <v>284</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>264</v>
+        <v>285</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>265</v>
+        <v>286</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>266</v>
+        <v>287</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>258</v>
+        <v>279</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>267</v>
+        <v>288</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>268</v>
+        <v>289</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>261</v>
+        <v>282</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>269</v>
+        <v>290</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>256</v>
+        <v>277</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>270</v>
+        <v>291</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>271</v>
+        <v>292</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>272</v>
+        <v>293</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>274</v>
+        <v>295</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>275</v>
+        <v>296</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>276</v>
+        <v>297</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="D11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>278</v>
+        <v>299</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>279</v>
+        <v>300</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>280</v>
+        <v>301</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>281</v>
+        <v>302</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>279</v>
+        <v>300</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>282</v>
+        <v>303</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>283</v>
+        <v>304</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>273</v>
+        <v>294</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>284</v>
+        <v>305</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>285</v>
+        <v>306</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>286</v>
+        <v>307</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>287</v>
+        <v>308</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>288</v>
+        <v>309</v>
       </c>
       <c r="D15" s="5"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>289</v>
+        <v>310</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>287</v>
+        <v>308</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>290</v>
+        <v>311</v>
       </c>
       <c r="D16" s="5"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>291</v>
+        <v>312</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>287</v>
+        <v>308</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>292</v>
+        <v>313</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>293</v>
+        <v>314</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>294</v>
+        <v>315</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>287</v>
+        <v>308</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>295</v>
+        <v>316</v>
       </c>
       <c r="D18" s="5"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>286</v>
+        <v>307</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>297</v>
+        <v>318</v>
       </c>
       <c r="D19" s="5"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>298</v>
+        <v>319</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>292</v>
+        <v>313</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>299</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>300</v>
+        <v>321</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>301</v>
+        <v>322</v>
       </c>
       <c r="D21" s="5"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>302</v>
+        <v>323</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>296</v>
+        <v>317</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>303</v>
+        <v>324</v>
       </c>
       <c r="D22" s="5"/>
     </row>
     <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>304</v>
+        <v>325</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>305</v>
+        <v>326</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>306</v>
+        <v>327</v>
       </c>
       <c r="D23" s="5"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>307</v>
+        <v>328</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>305</v>
+        <v>326</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>308</v>
+        <v>329</v>
       </c>
       <c r="D24" s="5"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>309</v>
+        <v>330</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>305</v>
+        <v>326</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>292</v>
+        <v>313</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>310</v>
+        <v>331</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>311</v>
+        <v>332</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>305</v>
+        <v>326</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>312</v>
+        <v>333</v>
       </c>
       <c r="D26" s="5"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>313</v>
+        <v>334</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>314</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>315</v>
+        <v>277</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>335</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>336</v>
       </c>
     </row>
   </sheetData>
@@ -3992,7 +4316,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -4003,7 +4327,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>316</v>
+        <v>337</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -4011,16 +4335,16 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>317</v>
+        <v>338</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>318</v>
+        <v>339</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>319</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4028,9 +4352,9 @@
         <v>1</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="C4" s="6"/>
+        <v>341</v>
+      </c>
+      <c r="C4" s="8"/>
       <c r="D4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4038,9 +4362,9 @@
         <v>2</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="C5" s="6"/>
+        <v>342</v>
+      </c>
+      <c r="C5" s="8"/>
       <c r="D5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4048,9 +4372,9 @@
         <v>3</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="C6" s="6"/>
+        <v>343</v>
+      </c>
+      <c r="C6" s="8"/>
       <c r="D6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4058,9 +4382,9 @@
         <v>4</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>323</v>
-      </c>
-      <c r="C7" s="6"/>
+        <v>344</v>
+      </c>
+      <c r="C7" s="8"/>
       <c r="D7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4068,9 +4392,9 @@
         <v>5</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>324</v>
-      </c>
-      <c r="C8" s="6"/>
+        <v>345</v>
+      </c>
+      <c r="C8" s="8"/>
       <c r="D8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4078,9 +4402,9 @@
         <v>6</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C9" s="6"/>
+        <v>346</v>
+      </c>
+      <c r="C9" s="8"/>
       <c r="D9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4088,9 +4412,9 @@
         <v>7</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="C10" s="6"/>
+        <v>347</v>
+      </c>
+      <c r="C10" s="8"/>
       <c r="D10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4098,9 +4422,9 @@
         <v>8</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="C11" s="6"/>
+        <v>348</v>
+      </c>
+      <c r="C11" s="8"/>
       <c r="D11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4108,9 +4432,9 @@
         <v>9</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="C12" s="6"/>
+        <v>349</v>
+      </c>
+      <c r="C12" s="8"/>
       <c r="D12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4118,20 +4442,40 @@
         <v>10</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="C13" s="6"/>
+        <v>350</v>
+      </c>
+      <c r="C13" s="8"/>
       <c r="D13" s="5"/>
     </row>
-    <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="n">
         <v>11</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="C14" s="6"/>
+        <v>351</v>
+      </c>
+      <c r="C14" s="8"/>
       <c r="D14" s="5"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="C15" s="8"/>
+      <c r="D15" s="5"/>
+    </row>
+    <row r="16" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="C16" s="8"/>
+      <c r="D16" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>